<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@422739232707efb5db901c48ed1c50af47bd5701 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-ACPTreatmentCodelist.xlsx
+++ b/ValueSet-ACPTreatmentCodelist.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include from SNOMED CT" r:id="rId4" sheetId="2"/>
+    <sheet name="Include from SNOWMED CT" r:id="rId4" sheetId="2"/>
     <sheet name="Include ValueSets" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-05-08T14:01:10+00:00</t>
+    <t>2024-05-13T07:35:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@50771bdd80c2552635d3f0952bfa9f94da51cf4a 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-ACPTreatmentCodelist.xlsx
+++ b/ValueSet-ACPTreatmentCodelist.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include from SNOWMED CT" r:id="rId4" sheetId="2"/>
+    <sheet name="Include from SNOMED CT" r:id="rId4" sheetId="2"/>
     <sheet name="Include ValueSets" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-05-16T14:46:55+00:00</t>
+    <t>2024-05-29T06:49:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@199cd1a4beb147008cf759cb1767c91597ecf949 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-ACPTreatmentCodelist.xlsx
+++ b/ValueSet-ACPTreatmentCodelist.xlsx
@@ -7,8 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include from SNOMED CT" r:id="rId4" sheetId="2"/>
-    <sheet name="Include ValueSets" r:id="rId5" sheetId="3"/>
+    <sheet name="Include #0" r:id="rId4" sheetId="2"/>
+    <sheet name="Include ValueSet #1" r:id="rId5" sheetId="3"/>
   </sheets>
 </workbook>
 </file>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-09-03T12:43:26+00:00</t>
+    <t>2024-09-10T15:15:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@c9f01d98f1ae92f9491763c8fad45073c8be0ca8 🚀
</commit_message>
<xml_diff>
--- a/ValueSet-ACPTreatmentCodelist.xlsx
+++ b/ValueSet-ACPTreatmentCodelist.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-11-28T08:25:00+00:00</t>
+    <t>2024-11-28T17:50:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -107,6 +107,12 @@
   </si>
   <si>
     <t>Concept</t>
+  </si>
+  <si>
+    <t>183452005</t>
+  </si>
+  <si>
+    <t>Emergency hospital admission (procedure)</t>
   </si>
   <si>
     <t>32485007</t>
@@ -413,7 +419,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.703125" customWidth="true"/>
@@ -457,15 +463,23 @@
         <v>37</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s" s="2">
         <v>39</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -484,12 +498,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>